<commit_message>
개발중 ( -ing )
</commit_message>
<xml_diff>
--- a/src/main/resources/doc/PONKIDS-테이블정의서_v3.9.xlsx
+++ b/src/main/resources/doc/PONKIDS-테이블정의서_v3.9.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/jjeoV/Desktop/jjeoV/2023/pioneerKids/workspace/ponkidsDev/ponkids/src/main/resources/doc/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{C32F18B3-6E7B-D64E-99FD-D3B9270E260D}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{B4765B6F-CB2E-EC47-B952-43DC6157B186}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-34200" yWindow="-2840" windowWidth="34200" windowHeight="21380" tabRatio="777" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="0" yWindow="860" windowWidth="34200" windowHeight="21380" tabRatio="777" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="테이블정의서" sheetId="26" r:id="rId1"/>
@@ -4697,6 +4697,9 @@
     <xf numFmtId="0" fontId="41" fillId="10" borderId="3" xfId="88" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
+    <xf numFmtId="0" fontId="37" fillId="0" borderId="3" xfId="97" quotePrefix="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
     <xf numFmtId="0" fontId="32" fillId="5" borderId="17" xfId="88" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
@@ -4704,9 +4707,6 @@
       <alignment horizontal="center" vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="32" fillId="5" borderId="19" xfId="88" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="37" fillId="0" borderId="3" xfId="97" quotePrefix="1" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
   </cellXfs>
@@ -5236,7 +5236,7 @@
     <col min="24" max="24" width="14.33203125" style="124" bestFit="1" customWidth="1"/>
     <col min="25" max="25" width="68.1640625" style="124" customWidth="1"/>
     <col min="26" max="26" width="40.83203125" style="124" bestFit="1" customWidth="1"/>
-    <col min="27" max="27" width="60.6640625" style="124" customWidth="1"/>
+    <col min="27" max="27" width="159.6640625" style="124" customWidth="1"/>
     <col min="28" max="28" width="41.5" style="124" customWidth="1"/>
     <col min="29" max="29" width="83.1640625" style="124" customWidth="1"/>
     <col min="30" max="30" width="80.6640625" style="124" customWidth="1"/>
@@ -5303,25 +5303,25 @@
       <c r="W2" s="40"/>
     </row>
     <row r="3" spans="1:35" s="41" customFormat="1" ht="25" customHeight="1">
-      <c r="A3" s="153"/>
-      <c r="B3" s="154"/>
-      <c r="C3" s="154"/>
-      <c r="D3" s="154"/>
-      <c r="E3" s="154"/>
-      <c r="F3" s="154"/>
-      <c r="G3" s="154"/>
-      <c r="H3" s="154"/>
-      <c r="I3" s="154"/>
-      <c r="J3" s="154"/>
-      <c r="K3" s="154"/>
-      <c r="L3" s="154"/>
-      <c r="M3" s="154"/>
-      <c r="N3" s="154"/>
-      <c r="O3" s="154"/>
-      <c r="P3" s="154"/>
-      <c r="Q3" s="154"/>
-      <c r="R3" s="154"/>
-      <c r="S3" s="155"/>
+      <c r="A3" s="154"/>
+      <c r="B3" s="155"/>
+      <c r="C3" s="155"/>
+      <c r="D3" s="155"/>
+      <c r="E3" s="155"/>
+      <c r="F3" s="155"/>
+      <c r="G3" s="155"/>
+      <c r="H3" s="155"/>
+      <c r="I3" s="155"/>
+      <c r="J3" s="155"/>
+      <c r="K3" s="155"/>
+      <c r="L3" s="155"/>
+      <c r="M3" s="155"/>
+      <c r="N3" s="155"/>
+      <c r="O3" s="155"/>
+      <c r="P3" s="155"/>
+      <c r="Q3" s="155"/>
+      <c r="R3" s="155"/>
+      <c r="S3" s="156"/>
       <c r="T3" s="132"/>
       <c r="U3" s="132"/>
       <c r="V3" s="133"/>
@@ -6706,7 +6706,7 @@
         <v/>
       </c>
       <c r="AB18" s="125" t="str">
-        <f t="shared" ref="AB18:AB22" si="12">IF(ISBLANK(T18),"","CREATE SEQUENCE "&amp;T18&amp;" START 100000;")</f>
+        <f t="shared" ref="AB18:AB21" si="12">IF(ISBLANK(T18),"","CREATE SEQUENCE "&amp;T18&amp;" START 100000;")</f>
         <v/>
       </c>
       <c r="AC18" s="125" t="str">
@@ -7994,7 +7994,7 @@
       <c r="Q33" s="119" t="s">
         <v>527</v>
       </c>
-      <c r="R33" s="156" t="s">
+      <c r="R33" s="153" t="s">
         <v>835</v>
       </c>
       <c r="S33" s="107" t="s">
@@ -8084,7 +8084,7 @@
         <v>706</v>
       </c>
       <c r="Q34" s="119"/>
-      <c r="R34" s="156" t="s">
+      <c r="R34" s="153" t="s">
         <v>836</v>
       </c>
       <c r="S34" s="107" t="s">

</xml_diff>